<commit_message>
for live at first
</commit_message>
<xml_diff>
--- a/fixtures/seed_data.xlsx
+++ b/fixtures/seed_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\feevert-pro\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06E1B94-FD12-4679-80C8-6F7F91CC82F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A8C01A8-F871-4755-8A67-DFA6770D02E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="16656" windowHeight="10680" firstSheet="14" activeTab="18" xr2:uid="{D15F9AC0-767E-4280-9552-DDD9367DD8A3}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="12684" windowHeight="10680" activeTab="2" xr2:uid="{D15F9AC0-767E-4280-9552-DDD9367DD8A3}"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="1" r:id="rId1"/>
@@ -4458,7 +4458,16 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="4"/>
+    <col min="1" max="1" width="18.44140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="4"/>
+    <col min="8" max="8" width="11.77734375" style="4" customWidth="1"/>
+    <col min="9" max="9" width="12.44140625" style="4" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="3" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
@@ -5941,7 +5950,13 @@
   <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="4"/>
+    <col min="1" max="1" width="26.5546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="21.109375" style="4" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" style="4" customWidth="1"/>
+    <col min="5" max="5" width="9" style="4" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
@@ -5970,7 +5985,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="216" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="102" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>21</v>
       </c>
@@ -5996,7 +6011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="91.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>25</v>
       </c>
@@ -6022,7 +6037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="106.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -6048,7 +6063,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="135.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>33</v>
       </c>
@@ -6074,7 +6089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="126.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
@@ -6100,7 +6115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>41</v>
       </c>
@@ -6126,7 +6141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>45</v>
       </c>
@@ -6152,7 +6167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="216" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="130.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>49</v>
       </c>
@@ -6178,7 +6193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="121.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>52</v>
       </c>
@@ -6204,7 +6219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="142.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>56</v>
       </c>
@@ -6215,7 +6230,7 @@
         <v>58</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="E11" s="4">
         <v>1</v>
@@ -6256,7 +6271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="216" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="126" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>64</v>
       </c>
@@ -6282,7 +6297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="140.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>68</v>
       </c>
@@ -6308,7 +6323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="273.60000000000002" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>72</v>
       </c>
@@ -6334,7 +6349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="88.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>76</v>
       </c>
@@ -6360,7 +6375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="95.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>80</v>
       </c>
@@ -6386,7 +6401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="103.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>84</v>
       </c>
@@ -6412,7 +6427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="216" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="128.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>88</v>
       </c>
@@ -6438,7 +6453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="108.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>91</v>
       </c>
@@ -6490,7 +6505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="117" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>99</v>
       </c>

</xml_diff>